<commit_message>
python script that generates xlsx/csv files and charts
</commit_message>
<xml_diff>
--- a/results/results.xlsx
+++ b/results/results.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -429,8 +429,10 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -456,22 +458,32 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>memory_mb</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>conflicts</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>decisions</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>propagations</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>memory_mb</t>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>conflicts_per_sec</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>propagations_per_sec</t>
         </is>
       </c>
     </row>
@@ -494,17 +506,23 @@
       <c r="D2" s="2" t="n">
         <v>1320.18</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E2" s="2" t="n">
+        <v>77.77</v>
+      </c>
+      <c r="F2" t="n">
         <v>42579409</v>
       </c>
-      <c r="F2" t="n">
+      <c r="G2" t="n">
         <v>46109306</v>
       </c>
-      <c r="G2" t="n">
+      <c r="H2" t="n">
         <v>4132859697</v>
       </c>
-      <c r="H2" s="2" t="n">
-        <v>77.77</v>
+      <c r="I2" s="2" t="n">
+        <v>32252.72993076701</v>
+      </c>
+      <c r="J2" s="2" t="n">
+        <v>3130527.425805572</v>
       </c>
     </row>
     <row r="3">
@@ -526,14 +544,20 @@
       <c r="D3" s="2" t="n">
         <v>26163</v>
       </c>
-      <c r="E3" t="n">
+      <c r="F3" t="n">
         <v>149754456</v>
       </c>
-      <c r="F3" t="n">
+      <c r="G3" t="n">
         <v>160844936</v>
       </c>
-      <c r="G3" t="n">
+      <c r="H3" t="n">
         <v>17052139761</v>
+      </c>
+      <c r="I3" s="2" t="n">
+        <v>5723.902304781562</v>
+      </c>
+      <c r="J3" s="2" t="n">
+        <v>651765.4611856438</v>
       </c>
     </row>
     <row r="4">
@@ -555,17 +579,23 @@
       <c r="D4" s="2" t="n">
         <v>237.889</v>
       </c>
-      <c r="E4" t="n">
+      <c r="E4" s="2" t="n">
+        <v>57.57</v>
+      </c>
+      <c r="F4" t="n">
         <v>5013163</v>
       </c>
-      <c r="F4" t="n">
+      <c r="G4" t="n">
         <v>6227714</v>
       </c>
-      <c r="G4" t="n">
+      <c r="H4" t="n">
         <v>485718708</v>
       </c>
-      <c r="H4" s="2" t="n">
-        <v>57.57</v>
+      <c r="I4" s="2" t="n">
+        <v>21073.53849904787</v>
+      </c>
+      <c r="J4" s="2" t="n">
+        <v>2041787.169646348</v>
       </c>
     </row>
     <row r="5">
@@ -587,14 +617,20 @@
       <c r="D5" s="2" t="n">
         <v>273.347</v>
       </c>
-      <c r="E5" t="n">
+      <c r="F5" t="n">
         <v>1483777</v>
       </c>
-      <c r="F5" t="n">
+      <c r="G5" t="n">
         <v>1885201</v>
       </c>
-      <c r="G5" t="n">
+      <c r="H5" t="n">
         <v>144246338</v>
+      </c>
+      <c r="I5" s="2" t="n">
+        <v>5428.181029972892</v>
+      </c>
+      <c r="J5" s="2" t="n">
+        <v>527704.1196720653</v>
       </c>
     </row>
   </sheetData>

</xml_diff>